<commit_message>
update profiles description ffe6cb38b3ce608fcc54d3f03aa3dd70fddaa710
</commit_message>
<xml_diff>
--- a/nr-update-pages/ig/StructureDefinition-FrRangeMedication.xlsx
+++ b/nr-update-pages/ig/StructureDefinition-FrRangeMedication.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-12-29T12:28:59+00:00</t>
+    <t>2025-12-29T12:57:50+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,7 +84,8 @@
     <t>Description</t>
   </si>
   <si>
-    <t>Range with low and high unit UCUM or EDQM codes if code is used</t>
+    <t>Range with low and high unit UCUM or EDQM codes if code is used
+Plage avec des unités UCUM ou EDQM si un code est utilisé.</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>